<commit_message>
Update Excel: headers azul, concepto/proveedor azul, ppto azul, real verde
</commit_message>
<xml_diff>
--- a/Reporte_Gastos_Tecnologia_Bolivar_2026.xlsx
+++ b/Reporte_Gastos_Tecnologia_Bolivar_2026.xlsx
@@ -51,8 +51,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002E5FA3"/>
+      <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
@@ -62,13 +61,8 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="002E5FA3"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="004A7FC1"/>
+      <color rgb="001A1A18"/>
       <sz val="9"/>
     </font>
     <font>
@@ -76,6 +70,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002E5FA3"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="10">
@@ -87,7 +87,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B3F6E"/>
+        <fgColor rgb="003C3C3B"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,7 +107,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A7FC1"/>
+        <fgColor rgb="000D7A5F"/>
       </patternFill>
     </fill>
     <fill>
@@ -117,7 +117,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00E8F5F1"/>
       </patternFill>
     </fill>
     <fill>
@@ -126,7 +126,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -136,16 +136,16 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="001B3F6E"/>
+        <color rgb="003C3C3B"/>
       </left>
       <right style="medium">
-        <color rgb="001B3F6E"/>
+        <color rgb="003C3C3B"/>
       </right>
       <top style="medium">
-        <color rgb="001B3F6E"/>
+        <color rgb="003C3C3B"/>
       </top>
       <bottom style="medium">
-        <color rgb="001B3F6E"/>
+        <color rgb="003C3C3B"/>
       </bottom>
     </border>
     <border>
@@ -178,23 +178,180 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="004A7FC1"/>
+        <color rgb="000D7A5F"/>
       </left>
       <right style="medium">
-        <color rgb="004A7FC1"/>
+        <color rgb="000D7A5F"/>
       </right>
       <top style="medium">
-        <color rgb="004A7FC1"/>
+        <color rgb="000D7A5F"/>
       </top>
       <bottom style="medium">
-        <color rgb="004A7FC1"/>
+        <color rgb="000D7A5F"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="003C3C3B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="003C3C3B"/>
+      </right>
+      <top style="medium">
+        <color rgb="003C3C3B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="003C3C3B"/>
+      </right>
+      <top style="medium">
+        <color rgb="003C3C3B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="003C3C3B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="003C3C3B"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="003C3C3B"/>
+      </left>
+      <right style="medium">
+        <color rgb="003C3C3B"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="003C3C3B"/>
+      </left>
+      <right style="medium">
+        <color rgb="003C3C3B"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="003C3C3B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="003C3C3B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="003C3C3B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -214,67 +371,88 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -637,7 +815,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002E5FA3"/>
+    <tabColor rgb="00C8722A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -681,6 +859,34 @@
           <t>INVERSIONES BOLÍVAR S.A. DE C.V.  ·  PRESUPUESTO ÁREA DE TECNOLOGÍA 2026</t>
         </is>
       </c>
+      <c r="B1" s="25" t="n"/>
+      <c r="C1" s="25" t="n"/>
+      <c r="D1" s="25" t="n"/>
+      <c r="E1" s="25" t="n"/>
+      <c r="F1" s="25" t="n"/>
+      <c r="G1" s="25" t="n"/>
+      <c r="H1" s="25" t="n"/>
+      <c r="I1" s="25" t="n"/>
+      <c r="J1" s="25" t="n"/>
+      <c r="K1" s="25" t="n"/>
+      <c r="L1" s="25" t="n"/>
+      <c r="M1" s="25" t="n"/>
+      <c r="N1" s="25" t="n"/>
+      <c r="O1" s="25" t="n"/>
+      <c r="P1" s="25" t="n"/>
+      <c r="Q1" s="25" t="n"/>
+      <c r="R1" s="25" t="n"/>
+      <c r="S1" s="25" t="n"/>
+      <c r="T1" s="25" t="n"/>
+      <c r="U1" s="25" t="n"/>
+      <c r="V1" s="25" t="n"/>
+      <c r="W1" s="25" t="n"/>
+      <c r="X1" s="25" t="n"/>
+      <c r="Y1" s="25" t="n"/>
+      <c r="Z1" s="25" t="n"/>
+      <c r="AA1" s="25" t="n"/>
+      <c r="AB1" s="25" t="n"/>
+      <c r="AC1" s="26" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -688,6 +894,34 @@
           <t>Seguimiento Presupuestal — Ppto vs Real por partida y proveedor</t>
         </is>
       </c>
+      <c r="B2" s="25" t="n"/>
+      <c r="C2" s="25" t="n"/>
+      <c r="D2" s="25" t="n"/>
+      <c r="E2" s="25" t="n"/>
+      <c r="F2" s="25" t="n"/>
+      <c r="G2" s="25" t="n"/>
+      <c r="H2" s="25" t="n"/>
+      <c r="I2" s="25" t="n"/>
+      <c r="J2" s="25" t="n"/>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+      <c r="M2" s="25" t="n"/>
+      <c r="N2" s="25" t="n"/>
+      <c r="O2" s="25" t="n"/>
+      <c r="P2" s="25" t="n"/>
+      <c r="Q2" s="25" t="n"/>
+      <c r="R2" s="25" t="n"/>
+      <c r="S2" s="25" t="n"/>
+      <c r="T2" s="25" t="n"/>
+      <c r="U2" s="25" t="n"/>
+      <c r="V2" s="25" t="n"/>
+      <c r="W2" s="25" t="n"/>
+      <c r="X2" s="25" t="n"/>
+      <c r="Y2" s="25" t="n"/>
+      <c r="Z2" s="25" t="n"/>
+      <c r="AA2" s="25" t="n"/>
+      <c r="AB2" s="25" t="n"/>
+      <c r="AC2" s="26" t="n"/>
     </row>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -695,15 +929,43 @@
           <t>Fuente: Intelisis ERP + PPTO 2026 Josué Ramírez  ·  28/05/2026</t>
         </is>
       </c>
+      <c r="B3" s="25" t="n"/>
+      <c r="C3" s="25" t="n"/>
+      <c r="D3" s="25" t="n"/>
+      <c r="E3" s="25" t="n"/>
+      <c r="F3" s="25" t="n"/>
+      <c r="G3" s="25" t="n"/>
+      <c r="H3" s="25" t="n"/>
+      <c r="I3" s="25" t="n"/>
+      <c r="J3" s="25" t="n"/>
+      <c r="K3" s="25" t="n"/>
+      <c r="L3" s="25" t="n"/>
+      <c r="M3" s="25" t="n"/>
+      <c r="N3" s="25" t="n"/>
+      <c r="O3" s="25" t="n"/>
+      <c r="P3" s="25" t="n"/>
+      <c r="Q3" s="25" t="n"/>
+      <c r="R3" s="25" t="n"/>
+      <c r="S3" s="25" t="n"/>
+      <c r="T3" s="25" t="n"/>
+      <c r="U3" s="25" t="n"/>
+      <c r="V3" s="25" t="n"/>
+      <c r="W3" s="25" t="n"/>
+      <c r="X3" s="25" t="n"/>
+      <c r="Y3" s="25" t="n"/>
+      <c r="Z3" s="25" t="n"/>
+      <c r="AA3" s="25" t="n"/>
+      <c r="AB3" s="25" t="n"/>
+      <c r="AC3" s="26" t="n"/>
     </row>
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="34" t="inlineStr">
         <is>
           <t>Comentario / Proveedor</t>
         </is>
@@ -713,61 +975,73 @@
           <t>Ene</t>
         </is>
       </c>
+      <c r="D5" s="26" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
+      <c r="F5" s="26" t="n"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
+      <c r="H5" s="26" t="n"/>
       <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Abr</t>
         </is>
       </c>
+      <c r="J5" s="26" t="n"/>
       <c r="K5" s="5" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
+      <c r="L5" s="26" t="n"/>
       <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
+      <c r="N5" s="26" t="n"/>
       <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
+      <c r="P5" s="26" t="n"/>
       <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>Ago</t>
         </is>
       </c>
+      <c r="R5" s="26" t="n"/>
       <c r="S5" s="5" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
+      <c r="T5" s="26" t="n"/>
       <c r="U5" s="5" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
+      <c r="V5" s="26" t="n"/>
       <c r="W5" s="5" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
+      <c r="X5" s="26" t="n"/>
       <c r="Y5" s="5" t="inlineStr">
         <is>
           <t>Dic</t>
         </is>
       </c>
+      <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="5" t="inlineStr">
         <is>
           <t>Total Ppto</t>
@@ -778,13 +1052,15 @@
           <t>Total Real</t>
         </is>
       </c>
-      <c r="AC5" s="4" t="inlineStr">
+      <c r="AC5" s="34" t="inlineStr">
         <is>
           <t>Cuenta</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="37" t="n"/>
+      <c r="B6" s="37" t="n"/>
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Ppto</t>
@@ -905,14 +1181,17 @@
           <t>Real</t>
         </is>
       </c>
+      <c r="AA6" s="27" t="n"/>
+      <c r="AB6" s="27" t="n"/>
+      <c r="AC6" s="27" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>ADM-LICENCIAS DE PROGRAMAS</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Intelisis (Grupo Octo)</t>
         </is>
@@ -981,70 +1260,70 @@
       <c r="AB7" s="13" t="n">
         <v>17500</v>
       </c>
-      <c r="AC7" s="14" t="inlineStr">
+      <c r="AC7" s="30" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>ADM-LICENCIAS DE PROGRAMAS</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="32" t="inlineStr">
         <is>
           <t>Licencia Fortigate</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n"/>
-      <c r="G8" s="17" t="n"/>
-      <c r="H8" s="17" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="11" t="n"/>
       <c r="I8" s="9" t="n">
         <v>5000</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>5000</v>
       </c>
-      <c r="K8" s="17" t="n"/>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="17" t="n"/>
-      <c r="N8" s="17" t="n"/>
-      <c r="O8" s="17" t="n"/>
-      <c r="P8" s="17" t="n"/>
-      <c r="Q8" s="17" t="n"/>
-      <c r="R8" s="17" t="n"/>
-      <c r="S8" s="17" t="n"/>
-      <c r="T8" s="17" t="n"/>
-      <c r="U8" s="17" t="n"/>
-      <c r="V8" s="17" t="n"/>
-      <c r="W8" s="17" t="n"/>
-      <c r="X8" s="17" t="n"/>
-      <c r="Y8" s="17" t="n"/>
-      <c r="Z8" s="17" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="11" t="n"/>
+      <c r="M8" s="15" t="n"/>
+      <c r="N8" s="11" t="n"/>
+      <c r="O8" s="15" t="n"/>
+      <c r="P8" s="11" t="n"/>
+      <c r="Q8" s="15" t="n"/>
+      <c r="R8" s="11" t="n"/>
+      <c r="S8" s="15" t="n"/>
+      <c r="T8" s="11" t="n"/>
+      <c r="U8" s="15" t="n"/>
+      <c r="V8" s="11" t="n"/>
+      <c r="W8" s="15" t="n"/>
+      <c r="X8" s="11" t="n"/>
+      <c r="Y8" s="15" t="n"/>
+      <c r="Z8" s="11" t="n"/>
       <c r="AA8" s="12" t="n">
         <v>5000</v>
       </c>
       <c r="AB8" s="13" t="n">
         <v>5000</v>
       </c>
-      <c r="AC8" s="18" t="inlineStr">
+      <c r="AC8" s="33" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>ADM-LICENCIAS DE PROGRAMAS</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>Laserfiche</t>
         </is>
@@ -1100,273 +1379,273 @@
       <c r="AA9" s="12" t="n">
         <v>6301.2</v>
       </c>
-      <c r="AB9" s="19" t="n"/>
-      <c r="AC9" s="14" t="inlineStr">
+      <c r="AB9" s="16" t="n"/>
+      <c r="AC9" s="30" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>ADM-LICENCIAS DE PROGRAMAS</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>Photoshop arquitectas</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="11" t="n"/>
       <c r="G10" s="9" t="n">
         <v>120</v>
       </c>
-      <c r="H10" s="17" t="n"/>
-      <c r="I10" s="17" t="n"/>
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="15" t="n"/>
       <c r="J10" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="K10" s="17" t="n"/>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="17" t="n"/>
-      <c r="N10" s="17" t="n"/>
-      <c r="O10" s="17" t="n"/>
-      <c r="P10" s="17" t="n"/>
-      <c r="Q10" s="17" t="n"/>
-      <c r="R10" s="17" t="n"/>
-      <c r="S10" s="17" t="n"/>
-      <c r="T10" s="17" t="n"/>
-      <c r="U10" s="17" t="n"/>
-      <c r="V10" s="17" t="n"/>
-      <c r="W10" s="17" t="n"/>
-      <c r="X10" s="17" t="n"/>
-      <c r="Y10" s="17" t="n"/>
-      <c r="Z10" s="17" t="n"/>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="11" t="n"/>
+      <c r="M10" s="15" t="n"/>
+      <c r="N10" s="11" t="n"/>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="11" t="n"/>
+      <c r="Q10" s="15" t="n"/>
+      <c r="R10" s="11" t="n"/>
+      <c r="S10" s="15" t="n"/>
+      <c r="T10" s="11" t="n"/>
+      <c r="U10" s="15" t="n"/>
+      <c r="V10" s="11" t="n"/>
+      <c r="W10" s="15" t="n"/>
+      <c r="X10" s="11" t="n"/>
+      <c r="Y10" s="15" t="n"/>
+      <c r="Z10" s="11" t="n"/>
       <c r="AA10" s="12" t="n">
         <v>120</v>
       </c>
       <c r="AB10" s="13" t="n">
         <v>110</v>
       </c>
-      <c r="AC10" s="18" t="inlineStr">
+      <c r="AC10" s="33" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>ADM-INTELIGENCIA ARTIFICIAL</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>OpenAI (múltiples usuarios)</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n"/>
+      <c r="C11" s="15" t="n"/>
       <c r="D11" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="E11" s="11" t="n"/>
+      <c r="E11" s="15" t="n"/>
       <c r="F11" s="10" t="n">
         <v>180</v>
       </c>
-      <c r="G11" s="11" t="n"/>
+      <c r="G11" s="15" t="n"/>
       <c r="H11" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="I11" s="11" t="n"/>
+      <c r="I11" s="15" t="n"/>
       <c r="J11" s="10" t="n">
         <v>145</v>
       </c>
-      <c r="K11" s="11" t="n"/>
+      <c r="K11" s="15" t="n"/>
       <c r="L11" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="M11" s="11" t="n"/>
+      <c r="M11" s="15" t="n"/>
       <c r="N11" s="11" t="n"/>
-      <c r="O11" s="11" t="n"/>
+      <c r="O11" s="15" t="n"/>
       <c r="P11" s="11" t="n"/>
-      <c r="Q11" s="11" t="n"/>
+      <c r="Q11" s="15" t="n"/>
       <c r="R11" s="11" t="n"/>
-      <c r="S11" s="11" t="n"/>
+      <c r="S11" s="15" t="n"/>
       <c r="T11" s="11" t="n"/>
-      <c r="U11" s="11" t="n"/>
+      <c r="U11" s="15" t="n"/>
       <c r="V11" s="11" t="n"/>
-      <c r="W11" s="11" t="n"/>
+      <c r="W11" s="15" t="n"/>
       <c r="X11" s="11" t="n"/>
-      <c r="Y11" s="11" t="n"/>
+      <c r="Y11" s="15" t="n"/>
       <c r="Z11" s="11" t="n"/>
-      <c r="AA11" s="20" t="n"/>
+      <c r="AA11" s="17" t="n"/>
       <c r="AB11" s="13" t="n">
         <v>530</v>
       </c>
-      <c r="AC11" s="14" t="inlineStr">
+      <c r="AC11" s="30" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>ADM-INTELIGENCIA ARTIFICIAL</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>HeyGen Technology</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="15" t="n"/>
       <c r="F12" s="10" t="n">
         <v>36.25</v>
       </c>
-      <c r="G12" s="17" t="n"/>
+      <c r="G12" s="15" t="n"/>
       <c r="H12" s="10" t="n">
         <v>36.25</v>
       </c>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="17" t="n"/>
-      <c r="K12" s="17" t="n"/>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="11" t="n"/>
+      <c r="K12" s="15" t="n"/>
       <c r="L12" s="10" t="n">
         <v>72.5</v>
       </c>
-      <c r="M12" s="17" t="n"/>
-      <c r="N12" s="17" t="n"/>
-      <c r="O12" s="17" t="n"/>
-      <c r="P12" s="17" t="n"/>
-      <c r="Q12" s="17" t="n"/>
-      <c r="R12" s="17" t="n"/>
-      <c r="S12" s="17" t="n"/>
-      <c r="T12" s="17" t="n"/>
-      <c r="U12" s="17" t="n"/>
-      <c r="V12" s="17" t="n"/>
-      <c r="W12" s="17" t="n"/>
-      <c r="X12" s="17" t="n"/>
-      <c r="Y12" s="17" t="n"/>
-      <c r="Z12" s="17" t="n"/>
-      <c r="AA12" s="20" t="n"/>
+      <c r="M12" s="15" t="n"/>
+      <c r="N12" s="11" t="n"/>
+      <c r="O12" s="15" t="n"/>
+      <c r="P12" s="11" t="n"/>
+      <c r="Q12" s="15" t="n"/>
+      <c r="R12" s="11" t="n"/>
+      <c r="S12" s="15" t="n"/>
+      <c r="T12" s="11" t="n"/>
+      <c r="U12" s="15" t="n"/>
+      <c r="V12" s="11" t="n"/>
+      <c r="W12" s="15" t="n"/>
+      <c r="X12" s="11" t="n"/>
+      <c r="Y12" s="15" t="n"/>
+      <c r="Z12" s="11" t="n"/>
+      <c r="AA12" s="17" t="n"/>
       <c r="AB12" s="13" t="n">
         <v>145</v>
       </c>
-      <c r="AC12" s="18" t="inlineStr">
+      <c r="AC12" s="33" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="28" t="inlineStr">
         <is>
           <t>ADM-INTELIGENCIA ARTIFICIAL</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>Anthropic (Claude)</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n"/>
+      <c r="C13" s="15" t="n"/>
       <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
+      <c r="E13" s="15" t="n"/>
       <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="G13" s="15" t="n"/>
       <c r="H13" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="I13" s="11" t="n"/>
+      <c r="I13" s="15" t="n"/>
       <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
+      <c r="K13" s="15" t="n"/>
       <c r="L13" s="11" t="n"/>
-      <c r="M13" s="11" t="n"/>
+      <c r="M13" s="15" t="n"/>
       <c r="N13" s="11" t="n"/>
-      <c r="O13" s="11" t="n"/>
+      <c r="O13" s="15" t="n"/>
       <c r="P13" s="11" t="n"/>
-      <c r="Q13" s="11" t="n"/>
+      <c r="Q13" s="15" t="n"/>
       <c r="R13" s="11" t="n"/>
-      <c r="S13" s="11" t="n"/>
+      <c r="S13" s="15" t="n"/>
       <c r="T13" s="11" t="n"/>
-      <c r="U13" s="11" t="n"/>
+      <c r="U13" s="15" t="n"/>
       <c r="V13" s="11" t="n"/>
-      <c r="W13" s="11" t="n"/>
+      <c r="W13" s="15" t="n"/>
       <c r="X13" s="11" t="n"/>
-      <c r="Y13" s="11" t="n"/>
+      <c r="Y13" s="15" t="n"/>
       <c r="Z13" s="11" t="n"/>
-      <c r="AA13" s="20" t="n"/>
+      <c r="AA13" s="17" t="n"/>
       <c r="AB13" s="13" t="n">
         <v>125</v>
       </c>
-      <c r="AC13" s="14" t="inlineStr">
+      <c r="AC13" s="30" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>ADM-INTELIGENCIA ARTIFICIAL</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>Moonflow LLC</t>
         </is>
       </c>
-      <c r="C14" s="17" t="n"/>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="17" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="15" t="n"/>
       <c r="F14" s="10" t="n">
         <v>149</v>
       </c>
-      <c r="G14" s="17" t="n"/>
+      <c r="G14" s="15" t="n"/>
       <c r="H14" s="10" t="n">
         <v>149</v>
       </c>
-      <c r="I14" s="17" t="n"/>
-      <c r="J14" s="17" t="n"/>
-      <c r="K14" s="17" t="n"/>
-      <c r="L14" s="17" t="n"/>
-      <c r="M14" s="17" t="n"/>
-      <c r="N14" s="17" t="n"/>
-      <c r="O14" s="17" t="n"/>
-      <c r="P14" s="17" t="n"/>
-      <c r="Q14" s="17" t="n"/>
-      <c r="R14" s="17" t="n"/>
-      <c r="S14" s="17" t="n"/>
-      <c r="T14" s="17" t="n"/>
-      <c r="U14" s="17" t="n"/>
-      <c r="V14" s="17" t="n"/>
-      <c r="W14" s="17" t="n"/>
-      <c r="X14" s="17" t="n"/>
-      <c r="Y14" s="17" t="n"/>
-      <c r="Z14" s="17" t="n"/>
-      <c r="AA14" s="20" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="11" t="n"/>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="11" t="n"/>
+      <c r="M14" s="15" t="n"/>
+      <c r="N14" s="11" t="n"/>
+      <c r="O14" s="15" t="n"/>
+      <c r="P14" s="11" t="n"/>
+      <c r="Q14" s="15" t="n"/>
+      <c r="R14" s="11" t="n"/>
+      <c r="S14" s="15" t="n"/>
+      <c r="T14" s="11" t="n"/>
+      <c r="U14" s="15" t="n"/>
+      <c r="V14" s="11" t="n"/>
+      <c r="W14" s="15" t="n"/>
+      <c r="X14" s="11" t="n"/>
+      <c r="Y14" s="15" t="n"/>
+      <c r="Z14" s="11" t="n"/>
+      <c r="AA14" s="17" t="n"/>
       <c r="AB14" s="13" t="n">
         <v>298</v>
       </c>
-      <c r="AC14" s="18" t="inlineStr">
+      <c r="AC14" s="33" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>ADM-INTELIGENCIA ARTIFICIAL</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="29" t="inlineStr">
         <is>
           <t>Licencias Copilot (ppto)</t>
         </is>
@@ -1422,20 +1701,20 @@
       <c r="AA15" s="12" t="n">
         <v>3000</v>
       </c>
-      <c r="AB15" s="19" t="n"/>
-      <c r="AC15" s="14" t="inlineStr">
+      <c r="AB15" s="16" t="n"/>
+      <c r="AC15" s="30" t="inlineStr">
         <is>
           <t>412010904</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>UDESA-SUSCRIPCIONES DE SOFTWARE</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="32" t="inlineStr">
         <is>
           <t>Azure (Data &amp; Graphics)</t>
         </is>
@@ -1461,160 +1740,160 @@
       <c r="I16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="J16" s="17" t="n"/>
+      <c r="J16" s="11" t="n"/>
       <c r="K16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="L16" s="17" t="n"/>
+      <c r="L16" s="11" t="n"/>
       <c r="M16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="N16" s="17" t="n"/>
+      <c r="N16" s="11" t="n"/>
       <c r="O16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="P16" s="17" t="n"/>
+      <c r="P16" s="11" t="n"/>
       <c r="Q16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="R16" s="17" t="n"/>
+      <c r="R16" s="11" t="n"/>
       <c r="S16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="T16" s="17" t="n"/>
+      <c r="T16" s="11" t="n"/>
       <c r="U16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="V16" s="17" t="n"/>
+      <c r="V16" s="11" t="n"/>
       <c r="W16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="X16" s="17" t="n"/>
+      <c r="X16" s="11" t="n"/>
       <c r="Y16" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="Z16" s="17" t="n"/>
+      <c r="Z16" s="11" t="n"/>
       <c r="AA16" s="12" t="n">
         <v>8400</v>
       </c>
       <c r="AB16" s="13" t="n">
         <v>2815.19</v>
       </c>
-      <c r="AC16" s="18" t="inlineStr">
+      <c r="AC16" s="33" t="inlineStr">
         <is>
           <t>412010905</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>UDESA-SUSCRIPCIONES DE SOFTWARE</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="29" t="inlineStr">
         <is>
           <t>Microsoft 365 IB</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n"/>
+      <c r="C17" s="15" t="n"/>
       <c r="D17" s="10" t="n">
         <v>161.88</v>
       </c>
-      <c r="E17" s="11" t="n"/>
+      <c r="E17" s="15" t="n"/>
       <c r="F17" s="10" t="n">
         <v>428.01</v>
       </c>
-      <c r="G17" s="11" t="n"/>
+      <c r="G17" s="15" t="n"/>
       <c r="H17" s="11" t="n"/>
-      <c r="I17" s="11" t="n"/>
+      <c r="I17" s="15" t="n"/>
       <c r="J17" s="10" t="n">
         <v>416.92</v>
       </c>
-      <c r="K17" s="11" t="n"/>
+      <c r="K17" s="15" t="n"/>
       <c r="L17" s="10" t="n">
         <v>178.78</v>
       </c>
-      <c r="M17" s="11" t="n"/>
+      <c r="M17" s="15" t="n"/>
       <c r="N17" s="11" t="n"/>
-      <c r="O17" s="11" t="n"/>
+      <c r="O17" s="15" t="n"/>
       <c r="P17" s="11" t="n"/>
-      <c r="Q17" s="11" t="n"/>
+      <c r="Q17" s="15" t="n"/>
       <c r="R17" s="11" t="n"/>
-      <c r="S17" s="11" t="n"/>
+      <c r="S17" s="15" t="n"/>
       <c r="T17" s="11" t="n"/>
-      <c r="U17" s="11" t="n"/>
+      <c r="U17" s="15" t="n"/>
       <c r="V17" s="11" t="n"/>
-      <c r="W17" s="11" t="n"/>
+      <c r="W17" s="15" t="n"/>
       <c r="X17" s="11" t="n"/>
-      <c r="Y17" s="11" t="n"/>
+      <c r="Y17" s="15" t="n"/>
       <c r="Z17" s="11" t="n"/>
-      <c r="AA17" s="20" t="n"/>
+      <c r="AA17" s="17" t="n"/>
       <c r="AB17" s="13" t="n">
         <v>1185.59</v>
       </c>
-      <c r="AC17" s="14" t="inlineStr">
+      <c r="AC17" s="30" t="inlineStr">
         <is>
           <t>412010905</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>UDESA-SUSCRIPCIONES DE SOFTWARE</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>Autodesk</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n"/>
-      <c r="D18" s="17" t="n"/>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="17" t="n"/>
-      <c r="G18" s="17" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="15" t="n"/>
       <c r="H18" s="10" t="n">
         <v>427.97</v>
       </c>
-      <c r="I18" s="17" t="n"/>
+      <c r="I18" s="15" t="n"/>
       <c r="J18" s="10" t="n">
         <v>1587.95</v>
       </c>
-      <c r="K18" s="17" t="n"/>
-      <c r="L18" s="17" t="n"/>
-      <c r="M18" s="17" t="n"/>
-      <c r="N18" s="17" t="n"/>
-      <c r="O18" s="17" t="n"/>
-      <c r="P18" s="17" t="n"/>
-      <c r="Q18" s="17" t="n"/>
-      <c r="R18" s="17" t="n"/>
-      <c r="S18" s="17" t="n"/>
-      <c r="T18" s="17" t="n"/>
-      <c r="U18" s="17" t="n"/>
-      <c r="V18" s="17" t="n"/>
-      <c r="W18" s="17" t="n"/>
-      <c r="X18" s="17" t="n"/>
-      <c r="Y18" s="17" t="n"/>
-      <c r="Z18" s="17" t="n"/>
-      <c r="AA18" s="20" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="11" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="11" t="n"/>
+      <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="11" t="n"/>
+      <c r="S18" s="15" t="n"/>
+      <c r="T18" s="11" t="n"/>
+      <c r="U18" s="15" t="n"/>
+      <c r="V18" s="11" t="n"/>
+      <c r="W18" s="15" t="n"/>
+      <c r="X18" s="11" t="n"/>
+      <c r="Y18" s="15" t="n"/>
+      <c r="Z18" s="11" t="n"/>
+      <c r="AA18" s="17" t="n"/>
       <c r="AB18" s="13" t="n">
         <v>2015.92</v>
       </c>
-      <c r="AC18" s="18" t="inlineStr">
+      <c r="AC18" s="33" t="inlineStr">
         <is>
           <t>412010905</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>UDESA-SUSCRIPCIONES DE SOFTWARE</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="29" t="inlineStr">
         <is>
           <t>GLPi (Inventario IT)</t>
         </is>
@@ -1681,19 +1960,19 @@
       <c r="AB19" s="13" t="n">
         <v>224.25</v>
       </c>
-      <c r="AC19" s="14" t="inlineStr">
+      <c r="AC19" s="30" t="inlineStr">
         <is>
           <t>412010905</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>ADM-COMUNICACIONES</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="32" t="inlineStr">
         <is>
           <t>Internet IB (Liberty Networks)</t>
         </is>
@@ -1731,50 +2010,50 @@
       <c r="M20" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="N20" s="17" t="n"/>
+      <c r="N20" s="11" t="n"/>
       <c r="O20" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="P20" s="17" t="n"/>
+      <c r="P20" s="11" t="n"/>
       <c r="Q20" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="R20" s="17" t="n"/>
+      <c r="R20" s="11" t="n"/>
       <c r="S20" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="T20" s="17" t="n"/>
+      <c r="T20" s="11" t="n"/>
       <c r="U20" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="V20" s="17" t="n"/>
+      <c r="V20" s="11" t="n"/>
       <c r="W20" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="X20" s="17" t="n"/>
+      <c r="X20" s="11" t="n"/>
       <c r="Y20" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="Z20" s="17" t="n"/>
+      <c r="Z20" s="11" t="n"/>
       <c r="AA20" s="12" t="n">
         <v>7200</v>
       </c>
       <c r="AB20" s="13" t="n">
         <v>3000</v>
       </c>
-      <c r="AC20" s="18" t="inlineStr">
+      <c r="AC20" s="33" t="inlineStr">
         <is>
           <t>412010701</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>UDESA-SOPORTE TÉCNICO TERCERIZADO</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="29" t="inlineStr">
         <is>
           <t>Técnico destacado KNK (Canizalez)</t>
         </is>
@@ -1843,25 +2122,25 @@
       <c r="AB21" s="13" t="n">
         <v>3928.6</v>
       </c>
-      <c r="AC21" s="14" t="inlineStr">
+      <c r="AC21" s="30" t="inlineStr">
         <is>
           <t>412011220</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="31" t="inlineStr">
         <is>
           <t>UDESA-SOPORTE TÉCNICO TERCERIZADO</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>Soporte visitas de campo (Cruz Treminio)</t>
         </is>
       </c>
-      <c r="C22" s="17" t="n"/>
-      <c r="D22" s="17" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="11" t="n"/>
       <c r="E22" s="9" t="n">
         <v>300</v>
       </c>
@@ -1883,59 +2162,59 @@
       <c r="K22" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="L22" s="17" t="n"/>
+      <c r="L22" s="11" t="n"/>
       <c r="M22" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="N22" s="17" t="n"/>
+      <c r="N22" s="11" t="n"/>
       <c r="O22" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="P22" s="17" t="n"/>
+      <c r="P22" s="11" t="n"/>
       <c r="Q22" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="R22" s="17" t="n"/>
+      <c r="R22" s="11" t="n"/>
       <c r="S22" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="T22" s="17" t="n"/>
+      <c r="T22" s="11" t="n"/>
       <c r="U22" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="V22" s="17" t="n"/>
+      <c r="V22" s="11" t="n"/>
       <c r="W22" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="X22" s="17" t="n"/>
+      <c r="X22" s="11" t="n"/>
       <c r="Y22" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="Z22" s="17" t="n"/>
+      <c r="Z22" s="11" t="n"/>
       <c r="AA22" s="12" t="n">
         <v>3300</v>
       </c>
       <c r="AB22" s="13" t="n">
         <v>1108.8</v>
       </c>
-      <c r="AC22" s="18" t="inlineStr">
+      <c r="AC22" s="33" t="inlineStr">
         <is>
           <t>412011220</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>ADM-MANT. MOBILIARIO Y EQUIPO</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="29" t="inlineStr">
         <is>
           <t>Mantenimiento impresores RICOH</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n"/>
+      <c r="C23" s="15" t="n"/>
       <c r="D23" s="11" t="n"/>
       <c r="E23" s="9" t="n">
         <v>150</v>
@@ -1993,85 +2272,85 @@
       <c r="AB23" s="13" t="n">
         <v>360</v>
       </c>
-      <c r="AC23" s="14" t="inlineStr">
+      <c r="AC23" s="30" t="inlineStr">
         <is>
           <t>412010602</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>ADM-MANT. MOBILIARIO Y EQUIPO</t>
         </is>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="32" t="inlineStr">
         <is>
           <t>Mantenimiento racks IB (Cruz Treminio)</t>
         </is>
       </c>
-      <c r="C24" s="17" t="n"/>
-      <c r="D24" s="17" t="n"/>
-      <c r="E24" s="17" t="n"/>
-      <c r="F24" s="17" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="11" t="n"/>
       <c r="G24" s="9" t="n">
         <v>140</v>
       </c>
       <c r="H24" s="10" t="n">
         <v>140</v>
       </c>
-      <c r="I24" s="17" t="n"/>
-      <c r="J24" s="17" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="11" t="n"/>
       <c r="K24" s="9" t="n">
         <v>140</v>
       </c>
-      <c r="L24" s="17" t="n"/>
+      <c r="L24" s="11" t="n"/>
       <c r="M24" s="9" t="n">
         <v>140</v>
       </c>
-      <c r="N24" s="17" t="n"/>
-      <c r="O24" s="17" t="n"/>
-      <c r="P24" s="17" t="n"/>
-      <c r="Q24" s="17" t="n"/>
-      <c r="R24" s="17" t="n"/>
+      <c r="N24" s="11" t="n"/>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="11" t="n"/>
+      <c r="Q24" s="15" t="n"/>
+      <c r="R24" s="11" t="n"/>
       <c r="S24" s="9" t="n">
         <v>140</v>
       </c>
-      <c r="T24" s="17" t="n"/>
-      <c r="U24" s="17" t="n"/>
-      <c r="V24" s="17" t="n"/>
-      <c r="W24" s="17" t="n"/>
-      <c r="X24" s="17" t="n"/>
+      <c r="T24" s="11" t="n"/>
+      <c r="U24" s="15" t="n"/>
+      <c r="V24" s="11" t="n"/>
+      <c r="W24" s="15" t="n"/>
+      <c r="X24" s="11" t="n"/>
       <c r="Y24" s="9" t="n">
         <v>140</v>
       </c>
-      <c r="Z24" s="17" t="n"/>
+      <c r="Z24" s="11" t="n"/>
       <c r="AA24" s="12" t="n">
         <v>700</v>
       </c>
       <c r="AB24" s="13" t="n">
         <v>140</v>
       </c>
-      <c r="AC24" s="18" t="inlineStr">
+      <c r="AC24" s="33" t="inlineStr">
         <is>
           <t>412010602</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>ADM-MANT. MOBILIARIO Y EQUIPO</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>Mantenimiento UPS IB (Cruz Treminio)</t>
         </is>
       </c>
-      <c r="C25" s="11" t="n"/>
+      <c r="C25" s="15" t="n"/>
       <c r="D25" s="11" t="n"/>
-      <c r="E25" s="11" t="n"/>
+      <c r="E25" s="15" t="n"/>
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="9" t="n">
         <v>100</v>
@@ -2079,25 +2358,25 @@
       <c r="H25" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="I25" s="11" t="n"/>
+      <c r="I25" s="15" t="n"/>
       <c r="J25" s="11" t="n"/>
-      <c r="K25" s="11" t="n"/>
+      <c r="K25" s="15" t="n"/>
       <c r="L25" s="11" t="n"/>
       <c r="M25" s="9" t="n">
         <v>100</v>
       </c>
       <c r="N25" s="11" t="n"/>
-      <c r="O25" s="11" t="n"/>
+      <c r="O25" s="15" t="n"/>
       <c r="P25" s="11" t="n"/>
-      <c r="Q25" s="11" t="n"/>
+      <c r="Q25" s="15" t="n"/>
       <c r="R25" s="11" t="n"/>
       <c r="S25" s="9" t="n">
         <v>100</v>
       </c>
       <c r="T25" s="11" t="n"/>
-      <c r="U25" s="11" t="n"/>
+      <c r="U25" s="15" t="n"/>
       <c r="V25" s="11" t="n"/>
-      <c r="W25" s="11" t="n"/>
+      <c r="W25" s="15" t="n"/>
       <c r="X25" s="11" t="n"/>
       <c r="Y25" s="9" t="n">
         <v>100</v>
@@ -2109,77 +2388,77 @@
       <c r="AB25" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="AC25" s="14" t="inlineStr">
+      <c r="AC25" s="30" t="inlineStr">
         <is>
           <t>412010602</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="31" t="inlineStr">
         <is>
           <t>ADM-MANT. MOBILIARIO Y EQUIPO</t>
         </is>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="32" t="inlineStr">
         <is>
           <t>Mantenimiento 4T (Cruz Treminio)</t>
         </is>
       </c>
-      <c r="C26" s="17" t="n"/>
-      <c r="D26" s="17" t="n"/>
-      <c r="E26" s="17" t="n"/>
-      <c r="F26" s="17" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="11" t="n"/>
       <c r="G26" s="9" t="n">
         <v>1900</v>
       </c>
       <c r="H26" s="10" t="n">
         <v>1889</v>
       </c>
-      <c r="I26" s="17" t="n"/>
-      <c r="J26" s="17" t="n"/>
-      <c r="K26" s="17" t="n"/>
-      <c r="L26" s="17" t="n"/>
-      <c r="M26" s="17" t="n"/>
-      <c r="N26" s="17" t="n"/>
-      <c r="O26" s="17" t="n"/>
-      <c r="P26" s="17" t="n"/>
-      <c r="Q26" s="17" t="n"/>
-      <c r="R26" s="17" t="n"/>
-      <c r="S26" s="17" t="n"/>
-      <c r="T26" s="17" t="n"/>
-      <c r="U26" s="17" t="n"/>
-      <c r="V26" s="17" t="n"/>
-      <c r="W26" s="17" t="n"/>
-      <c r="X26" s="17" t="n"/>
-      <c r="Y26" s="17" t="n"/>
-      <c r="Z26" s="17" t="n"/>
+      <c r="I26" s="15" t="n"/>
+      <c r="J26" s="11" t="n"/>
+      <c r="K26" s="15" t="n"/>
+      <c r="L26" s="11" t="n"/>
+      <c r="M26" s="15" t="n"/>
+      <c r="N26" s="11" t="n"/>
+      <c r="O26" s="15" t="n"/>
+      <c r="P26" s="11" t="n"/>
+      <c r="Q26" s="15" t="n"/>
+      <c r="R26" s="11" t="n"/>
+      <c r="S26" s="15" t="n"/>
+      <c r="T26" s="11" t="n"/>
+      <c r="U26" s="15" t="n"/>
+      <c r="V26" s="11" t="n"/>
+      <c r="W26" s="15" t="n"/>
+      <c r="X26" s="11" t="n"/>
+      <c r="Y26" s="15" t="n"/>
+      <c r="Z26" s="11" t="n"/>
       <c r="AA26" s="12" t="n">
         <v>1900</v>
       </c>
       <c r="AB26" s="13" t="n">
         <v>1889</v>
       </c>
-      <c r="AC26" s="18" t="inlineStr">
+      <c r="AC26" s="33" t="inlineStr">
         <is>
           <t>412010602</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="28" t="inlineStr">
         <is>
           <t>ADM-CONSUMIBLES FOTOCOPIADORA</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="29" t="inlineStr">
         <is>
           <t>Toner impresores</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n"/>
+      <c r="C27" s="15" t="n"/>
       <c r="D27" s="11" t="n"/>
-      <c r="E27" s="11" t="n"/>
+      <c r="E27" s="15" t="n"/>
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="9" t="n">
         <v>550</v>
@@ -2187,31 +2466,31 @@
       <c r="H27" s="10" t="n">
         <v>522</v>
       </c>
-      <c r="I27" s="11" t="n"/>
+      <c r="I27" s="15" t="n"/>
       <c r="J27" s="11" t="n"/>
       <c r="K27" s="9" t="n">
         <v>550</v>
       </c>
       <c r="L27" s="11" t="n"/>
-      <c r="M27" s="11" t="n"/>
+      <c r="M27" s="15" t="n"/>
       <c r="N27" s="11" t="n"/>
       <c r="O27" s="9" t="n">
         <v>550</v>
       </c>
       <c r="P27" s="11" t="n"/>
-      <c r="Q27" s="11" t="n"/>
+      <c r="Q27" s="15" t="n"/>
       <c r="R27" s="11" t="n"/>
       <c r="S27" s="9" t="n">
         <v>550</v>
       </c>
       <c r="T27" s="11" t="n"/>
-      <c r="U27" s="11" t="n"/>
+      <c r="U27" s="15" t="n"/>
       <c r="V27" s="11" t="n"/>
       <c r="W27" s="9" t="n">
         <v>550</v>
       </c>
       <c r="X27" s="11" t="n"/>
-      <c r="Y27" s="11" t="n"/>
+      <c r="Y27" s="15" t="n"/>
       <c r="Z27" s="11" t="n"/>
       <c r="AA27" s="12" t="n">
         <v>2750</v>
@@ -2219,70 +2498,70 @@
       <c r="AB27" s="13" t="n">
         <v>522</v>
       </c>
-      <c r="AC27" s="14" t="inlineStr">
+      <c r="AC27" s="30" t="inlineStr">
         <is>
           <t>412010906</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>ADM-CONSUMIBLES FOTOCOPIADORA</t>
         </is>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="32" t="inlineStr">
         <is>
           <t>Impresiones adicionales color</t>
         </is>
       </c>
-      <c r="C28" s="17" t="n"/>
-      <c r="D28" s="17" t="n"/>
-      <c r="E28" s="17" t="n"/>
-      <c r="F28" s="17" t="n"/>
-      <c r="G28" s="17" t="n"/>
-      <c r="H28" s="17" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="11" t="n"/>
       <c r="I28" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="J28" s="17" t="n"/>
-      <c r="K28" s="17" t="n"/>
-      <c r="L28" s="17" t="n"/>
-      <c r="M28" s="17" t="n"/>
-      <c r="N28" s="17" t="n"/>
+      <c r="J28" s="11" t="n"/>
+      <c r="K28" s="15" t="n"/>
+      <c r="L28" s="11" t="n"/>
+      <c r="M28" s="15" t="n"/>
+      <c r="N28" s="11" t="n"/>
       <c r="O28" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="P28" s="17" t="n"/>
-      <c r="Q28" s="17" t="n"/>
-      <c r="R28" s="17" t="n"/>
-      <c r="S28" s="17" t="n"/>
-      <c r="T28" s="17" t="n"/>
+      <c r="P28" s="11" t="n"/>
+      <c r="Q28" s="15" t="n"/>
+      <c r="R28" s="11" t="n"/>
+      <c r="S28" s="15" t="n"/>
+      <c r="T28" s="11" t="n"/>
       <c r="U28" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="V28" s="17" t="n"/>
-      <c r="W28" s="17" t="n"/>
-      <c r="X28" s="17" t="n"/>
-      <c r="Y28" s="17" t="n"/>
-      <c r="Z28" s="17" t="n"/>
+      <c r="V28" s="11" t="n"/>
+      <c r="W28" s="15" t="n"/>
+      <c r="X28" s="11" t="n"/>
+      <c r="Y28" s="15" t="n"/>
+      <c r="Z28" s="11" t="n"/>
       <c r="AA28" s="12" t="n">
         <v>1200</v>
       </c>
-      <c r="AB28" s="19" t="n"/>
-      <c r="AC28" s="18" t="inlineStr">
+      <c r="AB28" s="16" t="n"/>
+      <c r="AC28" s="33" t="inlineStr">
         <is>
           <t>412010906</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="28" t="inlineStr">
         <is>
           <t>ADM-MANT. PLANTA TELEFÓNICA</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="29" t="inlineStr">
         <is>
           <t>Mantenimiento planta (EBD / E-Business)</t>
         </is>
@@ -2293,9 +2572,9 @@
       <c r="D29" s="10" t="n">
         <v>335</v>
       </c>
-      <c r="E29" s="11" t="n"/>
+      <c r="E29" s="15" t="n"/>
       <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
+      <c r="G29" s="15" t="n"/>
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="9" t="n">
         <v>380</v>
@@ -2303,25 +2582,25 @@
       <c r="J29" s="10" t="n">
         <v>335</v>
       </c>
-      <c r="K29" s="11" t="n"/>
+      <c r="K29" s="15" t="n"/>
       <c r="L29" s="11" t="n"/>
-      <c r="M29" s="11" t="n"/>
+      <c r="M29" s="15" t="n"/>
       <c r="N29" s="11" t="n"/>
       <c r="O29" s="9" t="n">
         <v>380</v>
       </c>
       <c r="P29" s="11" t="n"/>
-      <c r="Q29" s="11" t="n"/>
+      <c r="Q29" s="15" t="n"/>
       <c r="R29" s="11" t="n"/>
-      <c r="S29" s="11" t="n"/>
+      <c r="S29" s="15" t="n"/>
       <c r="T29" s="11" t="n"/>
       <c r="U29" s="9" t="n">
         <v>380</v>
       </c>
       <c r="V29" s="11" t="n"/>
-      <c r="W29" s="11" t="n"/>
+      <c r="W29" s="15" t="n"/>
       <c r="X29" s="11" t="n"/>
-      <c r="Y29" s="11" t="n"/>
+      <c r="Y29" s="15" t="n"/>
       <c r="Z29" s="11" t="n"/>
       <c r="AA29" s="12" t="n">
         <v>1520</v>
@@ -2329,179 +2608,180 @@
       <c r="AB29" s="13" t="n">
         <v>670</v>
       </c>
-      <c r="AC29" s="14" t="inlineStr">
+      <c r="AC29" s="30" t="inlineStr">
         <is>
           <t>412010605</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="31" t="inlineStr">
         <is>
           <t>UDESA-SERVICIOS DE TECNOLOGÍA</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="32" t="inlineStr">
         <is>
           <t>Ilumi Data</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
-      <c r="E30" s="17" t="n"/>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="15" t="n"/>
       <c r="F30" s="10" t="n">
         <v>769.92</v>
       </c>
-      <c r="G30" s="17" t="n"/>
+      <c r="G30" s="15" t="n"/>
       <c r="H30" s="10" t="n">
         <v>343.79</v>
       </c>
-      <c r="I30" s="17" t="n"/>
-      <c r="J30" s="17" t="n"/>
-      <c r="K30" s="17" t="n"/>
-      <c r="L30" s="17" t="n"/>
-      <c r="M30" s="17" t="n"/>
-      <c r="N30" s="17" t="n"/>
-      <c r="O30" s="17" t="n"/>
-      <c r="P30" s="17" t="n"/>
-      <c r="Q30" s="17" t="n"/>
-      <c r="R30" s="17" t="n"/>
-      <c r="S30" s="17" t="n"/>
-      <c r="T30" s="17" t="n"/>
-      <c r="U30" s="17" t="n"/>
-      <c r="V30" s="17" t="n"/>
-      <c r="W30" s="17" t="n"/>
-      <c r="X30" s="17" t="n"/>
-      <c r="Y30" s="17" t="n"/>
-      <c r="Z30" s="17" t="n"/>
-      <c r="AA30" s="20" t="n"/>
+      <c r="I30" s="15" t="n"/>
+      <c r="J30" s="11" t="n"/>
+      <c r="K30" s="15" t="n"/>
+      <c r="L30" s="11" t="n"/>
+      <c r="M30" s="15" t="n"/>
+      <c r="N30" s="11" t="n"/>
+      <c r="O30" s="15" t="n"/>
+      <c r="P30" s="11" t="n"/>
+      <c r="Q30" s="15" t="n"/>
+      <c r="R30" s="11" t="n"/>
+      <c r="S30" s="15" t="n"/>
+      <c r="T30" s="11" t="n"/>
+      <c r="U30" s="15" t="n"/>
+      <c r="V30" s="11" t="n"/>
+      <c r="W30" s="15" t="n"/>
+      <c r="X30" s="11" t="n"/>
+      <c r="Y30" s="15" t="n"/>
+      <c r="Z30" s="11" t="n"/>
+      <c r="AA30" s="17" t="n"/>
       <c r="AB30" s="13" t="n">
         <v>1113.71</v>
       </c>
-      <c r="AC30" s="18" t="inlineStr">
+      <c r="AC30" s="33" t="inlineStr">
         <is>
           <t>412011220</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="28" t="inlineStr">
         <is>
           <t>UDESA-SERVICIOS DE TECNOLOGÍA</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="29" t="inlineStr">
         <is>
           <t>Servicios tecnología JMTELCOM/Cruz T.</t>
         </is>
       </c>
-      <c r="C31" s="11" t="n"/>
+      <c r="C31" s="15" t="n"/>
       <c r="D31" s="11" t="n"/>
-      <c r="E31" s="11" t="n"/>
+      <c r="E31" s="15" t="n"/>
       <c r="F31" s="11" t="n"/>
-      <c r="G31" s="11" t="n"/>
+      <c r="G31" s="15" t="n"/>
       <c r="H31" s="11" t="n"/>
-      <c r="I31" s="11" t="n"/>
+      <c r="I31" s="15" t="n"/>
       <c r="J31" s="10" t="n">
         <v>7409.64</v>
       </c>
-      <c r="K31" s="11" t="n"/>
+      <c r="K31" s="15" t="n"/>
       <c r="L31" s="11" t="n"/>
-      <c r="M31" s="11" t="n"/>
+      <c r="M31" s="15" t="n"/>
       <c r="N31" s="11" t="n"/>
-      <c r="O31" s="11" t="n"/>
+      <c r="O31" s="15" t="n"/>
       <c r="P31" s="11" t="n"/>
-      <c r="Q31" s="11" t="n"/>
+      <c r="Q31" s="15" t="n"/>
       <c r="R31" s="11" t="n"/>
-      <c r="S31" s="11" t="n"/>
+      <c r="S31" s="15" t="n"/>
       <c r="T31" s="11" t="n"/>
-      <c r="U31" s="11" t="n"/>
+      <c r="U31" s="15" t="n"/>
       <c r="V31" s="11" t="n"/>
-      <c r="W31" s="11" t="n"/>
+      <c r="W31" s="15" t="n"/>
       <c r="X31" s="11" t="n"/>
-      <c r="Y31" s="11" t="n"/>
+      <c r="Y31" s="15" t="n"/>
       <c r="Z31" s="11" t="n"/>
-      <c r="AA31" s="20" t="n"/>
+      <c r="AA31" s="17" t="n"/>
       <c r="AB31" s="13" t="n">
         <v>7409.64</v>
       </c>
-      <c r="AC31" s="14" t="inlineStr">
+      <c r="AC31" s="30" t="inlineStr">
         <is>
           <t>412011220</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="21" t="inlineStr">
+      <c r="A32" s="35" t="inlineStr">
         <is>
           <t>TOTAL GENERAL — 25 partidas</t>
         </is>
       </c>
-      <c r="C32" s="22" t="n">
+      <c r="B32" s="38" t="n"/>
+      <c r="C32" s="19" t="n">
         <v>7500.1</v>
       </c>
-      <c r="D32" s="23" t="n">
+      <c r="D32" s="20" t="n">
         <v>6394.89</v>
       </c>
-      <c r="E32" s="22" t="n">
+      <c r="E32" s="19" t="n">
         <v>7570.1</v>
       </c>
-      <c r="F32" s="23" t="n">
+      <c r="F32" s="20" t="n">
         <v>7885.51</v>
       </c>
-      <c r="G32" s="22" t="n">
+      <c r="G32" s="19" t="n">
         <v>10380.1</v>
       </c>
-      <c r="H32" s="23" t="n">
+      <c r="H32" s="20" t="n">
         <v>10429.83</v>
       </c>
-      <c r="I32" s="22" t="n">
+      <c r="I32" s="19" t="n">
         <v>13350.1</v>
       </c>
-      <c r="J32" s="23" t="n">
+      <c r="J32" s="20" t="n">
         <v>20318.47</v>
       </c>
-      <c r="K32" s="22" t="n">
+      <c r="K32" s="19" t="n">
         <v>8260.1</v>
       </c>
-      <c r="L32" s="23" t="n">
+      <c r="L32" s="20" t="n">
         <v>5162</v>
       </c>
-      <c r="M32" s="22" t="n">
+      <c r="M32" s="19" t="n">
         <v>7810.1</v>
       </c>
-      <c r="N32" s="24" t="n"/>
-      <c r="O32" s="22" t="n">
+      <c r="N32" s="21" t="n"/>
+      <c r="O32" s="19" t="n">
         <v>8900.1</v>
       </c>
-      <c r="P32" s="24" t="n"/>
-      <c r="Q32" s="22" t="n">
+      <c r="P32" s="21" t="n"/>
+      <c r="Q32" s="19" t="n">
         <v>7570.1</v>
       </c>
-      <c r="R32" s="24" t="n"/>
-      <c r="S32" s="22" t="n">
+      <c r="R32" s="21" t="n"/>
+      <c r="S32" s="19" t="n">
         <v>8360.1</v>
       </c>
-      <c r="T32" s="24" t="n"/>
-      <c r="U32" s="22" t="n">
+      <c r="T32" s="21" t="n"/>
+      <c r="U32" s="19" t="n">
         <v>8350.1</v>
       </c>
-      <c r="V32" s="24" t="n"/>
-      <c r="W32" s="22" t="n">
+      <c r="V32" s="21" t="n"/>
+      <c r="W32" s="19" t="n">
         <v>8120.1</v>
       </c>
-      <c r="X32" s="24" t="n"/>
-      <c r="Y32" s="22" t="n">
+      <c r="X32" s="21" t="n"/>
+      <c r="Y32" s="19" t="n">
         <v>7810.1</v>
       </c>
-      <c r="Z32" s="24" t="n"/>
-      <c r="AA32" s="25" t="n">
+      <c r="Z32" s="21" t="n"/>
+      <c r="AA32" s="22" t="n">
         <v>103981.2</v>
       </c>
-      <c r="AB32" s="26" t="n">
+      <c r="AB32" s="23" t="n">
         <v>50190.7</v>
       </c>
-      <c r="AC32" s="27" t="n"/>
+      <c r="AC32" s="36" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="21">

</xml_diff>

<commit_message>
FINAL: 27 partidas valores exactos jefe
</commit_message>
<xml_diff>
--- a/Reporte_Gastos_Tecnologia_Bolivar_2026.xlsx
+++ b/Reporte_Gastos_Tecnologia_Bolivar_2026.xlsx
@@ -121,7 +121,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -185,11 +185,88 @@
         <color rgb="000D7A5F"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -267,6 +344,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -673,6 +753,34 @@
           <t>INVERSIONES BOLÍVAR S.A. DE C.V.  ·  PRESUPUESTO ÁREA DE TECNOLOGÍA 2026</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="27" t="n"/>
+      <c r="K1" s="27" t="n"/>
+      <c r="L1" s="27" t="n"/>
+      <c r="M1" s="27" t="n"/>
+      <c r="N1" s="27" t="n"/>
+      <c r="O1" s="27" t="n"/>
+      <c r="P1" s="27" t="n"/>
+      <c r="Q1" s="27" t="n"/>
+      <c r="R1" s="27" t="n"/>
+      <c r="S1" s="27" t="n"/>
+      <c r="T1" s="27" t="n"/>
+      <c r="U1" s="27" t="n"/>
+      <c r="V1" s="27" t="n"/>
+      <c r="W1" s="27" t="n"/>
+      <c r="X1" s="27" t="n"/>
+      <c r="Y1" s="27" t="n"/>
+      <c r="Z1" s="27" t="n"/>
+      <c r="AA1" s="27" t="n"/>
+      <c r="AB1" s="27" t="n"/>
+      <c r="AC1" s="28" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -680,6 +788,34 @@
           <t>Seguimiento Presupuestal — Ppto vs Real por partida y proveedor</t>
         </is>
       </c>
+      <c r="B2" s="27" t="n"/>
+      <c r="C2" s="27" t="n"/>
+      <c r="D2" s="27" t="n"/>
+      <c r="E2" s="27" t="n"/>
+      <c r="F2" s="27" t="n"/>
+      <c r="G2" s="27" t="n"/>
+      <c r="H2" s="27" t="n"/>
+      <c r="I2" s="27" t="n"/>
+      <c r="J2" s="27" t="n"/>
+      <c r="K2" s="27" t="n"/>
+      <c r="L2" s="27" t="n"/>
+      <c r="M2" s="27" t="n"/>
+      <c r="N2" s="27" t="n"/>
+      <c r="O2" s="27" t="n"/>
+      <c r="P2" s="27" t="n"/>
+      <c r="Q2" s="27" t="n"/>
+      <c r="R2" s="27" t="n"/>
+      <c r="S2" s="27" t="n"/>
+      <c r="T2" s="27" t="n"/>
+      <c r="U2" s="27" t="n"/>
+      <c r="V2" s="27" t="n"/>
+      <c r="W2" s="27" t="n"/>
+      <c r="X2" s="27" t="n"/>
+      <c r="Y2" s="27" t="n"/>
+      <c r="Z2" s="27" t="n"/>
+      <c r="AA2" s="27" t="n"/>
+      <c r="AB2" s="27" t="n"/>
+      <c r="AC2" s="28" t="n"/>
     </row>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -687,6 +823,34 @@
           <t>Fuente: Intelisis ERP + PPTO 2026  ·  28/05/2026</t>
         </is>
       </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="27" t="n"/>
+      <c r="J3" s="27" t="n"/>
+      <c r="K3" s="27" t="n"/>
+      <c r="L3" s="27" t="n"/>
+      <c r="M3" s="27" t="n"/>
+      <c r="N3" s="27" t="n"/>
+      <c r="O3" s="27" t="n"/>
+      <c r="P3" s="27" t="n"/>
+      <c r="Q3" s="27" t="n"/>
+      <c r="R3" s="27" t="n"/>
+      <c r="S3" s="27" t="n"/>
+      <c r="T3" s="27" t="n"/>
+      <c r="U3" s="27" t="n"/>
+      <c r="V3" s="27" t="n"/>
+      <c r="W3" s="27" t="n"/>
+      <c r="X3" s="27" t="n"/>
+      <c r="Y3" s="27" t="n"/>
+      <c r="Z3" s="27" t="n"/>
+      <c r="AA3" s="27" t="n"/>
+      <c r="AB3" s="27" t="n"/>
+      <c r="AC3" s="28" t="n"/>
     </row>
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="20" customHeight="1">
@@ -705,61 +869,73 @@
           <t>Ene</t>
         </is>
       </c>
+      <c r="D5" s="28" t="n"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
+      <c r="F5" s="28" t="n"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
+      <c r="H5" s="28" t="n"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Abr</t>
         </is>
       </c>
+      <c r="J5" s="28" t="n"/>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
+      <c r="L5" s="28" t="n"/>
       <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
+      <c r="N5" s="28" t="n"/>
       <c r="O5" s="4" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
+      <c r="P5" s="28" t="n"/>
       <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>Ago</t>
         </is>
       </c>
+      <c r="R5" s="28" t="n"/>
       <c r="S5" s="4" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
+      <c r="T5" s="28" t="n"/>
       <c r="U5" s="4" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
+      <c r="V5" s="28" t="n"/>
       <c r="W5" s="4" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
+      <c r="X5" s="28" t="n"/>
       <c r="Y5" s="4" t="inlineStr">
         <is>
           <t>Dic</t>
         </is>
       </c>
+      <c r="Z5" s="28" t="n"/>
       <c r="AA5" s="4" t="inlineStr">
         <is>
           <t>Total Ppto</t>
@@ -777,6 +953,8 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="29" t="n"/>
+      <c r="B6" s="29" t="n"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Ppto</t>
@@ -897,6 +1075,9 @@
           <t>Real</t>
         </is>
       </c>
+      <c r="AA6" s="29" t="n"/>
+      <c r="AB6" s="29" t="n"/>
+      <c r="AC6" s="29" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -996,13 +1177,13 @@
       <c r="F8" s="10" t="n"/>
       <c r="G8" s="16" t="n"/>
       <c r="H8" s="10" t="n"/>
-      <c r="I8" s="16" t="n"/>
+      <c r="I8" s="8" t="n">
+        <v>5000</v>
+      </c>
       <c r="J8" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="K8" s="8" t="n">
-        <v>5000</v>
-      </c>
+      <c r="K8" s="16" t="n"/>
       <c r="L8" s="10" t="n"/>
       <c r="M8" s="16" t="n"/>
       <c r="N8" s="10" t="n"/>
@@ -1265,35 +1446,31 @@
         <v>72.5</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="N12" s="10" t="n"/>
       <c r="O12" s="8" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="P12" s="10" t="n"/>
       <c r="Q12" s="8" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="R12" s="10" t="n"/>
       <c r="S12" s="8" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="T12" s="10" t="n"/>
       <c r="U12" s="8" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="V12" s="10" t="n"/>
-      <c r="W12" s="8" t="n">
-        <v>99</v>
-      </c>
+      <c r="W12" s="16" t="n"/>
       <c r="X12" s="10" t="n"/>
-      <c r="Y12" s="8" t="n">
-        <v>99</v>
-      </c>
+      <c r="Y12" s="16" t="n"/>
       <c r="Z12" s="10" t="n"/>
       <c r="AA12" s="11" t="n">
-        <v>1173</v>
+        <v>900</v>
       </c>
       <c r="AB12" s="12" t="n">
         <v>145</v>
@@ -1640,11 +1817,15 @@
       <c r="T18" s="10" t="n"/>
       <c r="U18" s="16" t="n"/>
       <c r="V18" s="10" t="n"/>
-      <c r="W18" s="16" t="n"/>
+      <c r="W18" s="8" t="n">
+        <v>36000</v>
+      </c>
       <c r="X18" s="10" t="n"/>
       <c r="Y18" s="16" t="n"/>
       <c r="Z18" s="10" t="n"/>
-      <c r="AA18" s="19" t="n"/>
+      <c r="AA18" s="11" t="n">
+        <v>36000</v>
+      </c>
       <c r="AB18" s="12" t="n">
         <v>2015.92</v>
       </c>
@@ -2064,7 +2245,9 @@
       <c r="D24" s="10" t="n"/>
       <c r="E24" s="16" t="n"/>
       <c r="F24" s="10" t="n"/>
-      <c r="G24" s="16" t="n"/>
+      <c r="G24" s="8" t="n">
+        <v>140</v>
+      </c>
       <c r="H24" s="9" t="n">
         <v>140</v>
       </c>
@@ -2074,9 +2257,7 @@
         <v>140</v>
       </c>
       <c r="L24" s="10" t="n"/>
-      <c r="M24" s="8" t="n">
-        <v>140</v>
-      </c>
+      <c r="M24" s="16" t="n"/>
       <c r="N24" s="10" t="n"/>
       <c r="O24" s="16" t="n"/>
       <c r="P24" s="10" t="n"/>
@@ -2088,17 +2269,17 @@
       <c r="T24" s="10" t="n"/>
       <c r="U24" s="16" t="n"/>
       <c r="V24" s="10" t="n"/>
-      <c r="W24" s="16" t="n"/>
+      <c r="W24" s="8" t="n">
+        <v>140</v>
+      </c>
       <c r="X24" s="10" t="n"/>
-      <c r="Y24" s="8" t="n">
-        <v>140</v>
-      </c>
+      <c r="Y24" s="16" t="n"/>
       <c r="Z24" s="10" t="n"/>
       <c r="AA24" s="11" t="n">
         <v>560</v>
       </c>
       <c r="AB24" s="12" t="n">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="AC24" s="17" t="inlineStr">
         <is>
@@ -2140,19 +2321,19 @@
       <c r="Q25" s="16" t="n"/>
       <c r="R25" s="10" t="n"/>
       <c r="S25" s="8" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="T25" s="10" t="n"/>
       <c r="U25" s="16" t="n"/>
       <c r="V25" s="10" t="n"/>
-      <c r="W25" s="16" t="n"/>
+      <c r="W25" s="8" t="n">
+        <v>100</v>
+      </c>
       <c r="X25" s="10" t="n"/>
-      <c r="Y25" s="8" t="n">
-        <v>100</v>
-      </c>
+      <c r="Y25" s="16" t="n"/>
       <c r="Z25" s="10" t="n"/>
       <c r="AA25" s="11" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AB25" s="12" t="n">
         <v>100</v>
@@ -2416,7 +2597,9 @@
           <t>Impresiones adicionales color</t>
         </is>
       </c>
-      <c r="C30" s="16" t="n"/>
+      <c r="C30" s="8" t="n">
+        <v>400</v>
+      </c>
       <c r="D30" s="10" t="n"/>
       <c r="E30" s="16" t="n"/>
       <c r="F30" s="10" t="n"/>
@@ -2447,7 +2630,7 @@
       <c r="Y30" s="16" t="n"/>
       <c r="Z30" s="10" t="n"/>
       <c r="AA30" s="11" t="n">
-        <v>1200</v>
+        <v>1600</v>
       </c>
       <c r="AB30" s="18" t="n"/>
       <c r="AC30" s="17" t="inlineStr">
@@ -2612,15 +2795,11 @@
       <c r="E33" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="F33" s="9" t="n">
-        <v>769.92</v>
-      </c>
+      <c r="F33" s="10" t="n"/>
       <c r="G33" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="H33" s="9" t="n">
-        <v>343.79</v>
-      </c>
+      <c r="H33" s="10" t="n"/>
       <c r="I33" s="8" t="n">
         <v>400</v>
       </c>
@@ -2663,7 +2842,7 @@
         <v>4800</v>
       </c>
       <c r="AB33" s="12" t="n">
-        <v>8523.35</v>
+        <v>7409.64</v>
       </c>
       <c r="AC33" s="13" t="inlineStr">
         <is>
@@ -2677,8 +2856,9 @@
           <t>TOTAL GENERAL — 27 partidas</t>
         </is>
       </c>
+      <c r="B34" s="28" t="n"/>
       <c r="C34" s="21" t="n">
-        <v>9549.1</v>
+        <v>9949.1</v>
       </c>
       <c r="D34" s="22" t="n">
         <v>6464.65</v>
@@ -2687,59 +2867,59 @@
         <v>8619.1</v>
       </c>
       <c r="F34" s="22" t="n">
-        <v>8175.75</v>
+        <v>7405.83</v>
       </c>
       <c r="G34" s="21" t="n">
-        <v>11929.1</v>
+        <v>12069.1</v>
       </c>
       <c r="H34" s="22" t="n">
-        <v>11179.95</v>
+        <v>10696.16</v>
       </c>
       <c r="I34" s="21" t="n">
-        <v>9399.1</v>
+        <v>14399.1</v>
       </c>
       <c r="J34" s="22" t="n">
         <v>20532.59</v>
       </c>
       <c r="K34" s="21" t="n">
-        <v>14294.1</v>
+        <v>9294.1</v>
       </c>
       <c r="L34" s="22" t="n">
         <v>5237</v>
       </c>
       <c r="M34" s="21" t="n">
-        <v>8859.1</v>
+        <v>8704.1</v>
       </c>
       <c r="N34" s="23" t="n"/>
       <c r="O34" s="21" t="n">
-        <v>9949.1</v>
+        <v>9934.1</v>
       </c>
       <c r="P34" s="23" t="n"/>
       <c r="Q34" s="21" t="n">
-        <v>8619.1</v>
+        <v>8604.1</v>
       </c>
       <c r="R34" s="23" t="n"/>
       <c r="S34" s="21" t="n">
-        <v>9409.1</v>
+        <v>9494.1</v>
       </c>
       <c r="T34" s="23" t="n"/>
       <c r="U34" s="21" t="n">
-        <v>9399.1</v>
+        <v>9384.1</v>
       </c>
       <c r="V34" s="23" t="n"/>
       <c r="W34" s="21" t="n">
-        <v>9169.1</v>
+        <v>45310.1</v>
       </c>
       <c r="X34" s="23" t="n"/>
       <c r="Y34" s="21" t="n">
-        <v>8859.1</v>
+        <v>8520.1</v>
       </c>
       <c r="Z34" s="23" t="n"/>
       <c r="AA34" s="24" t="n">
-        <v>118054.2</v>
+        <v>154281.2</v>
       </c>
       <c r="AB34" s="25" t="n">
-        <v>51589.94</v>
+        <v>50336.23</v>
       </c>
       <c r="AC34" s="26" t="n"/>
     </row>

</xml_diff>

<commit_message>
Fix: ChatGPT Plus en UDESA-Suscripciones, valores Ene=60 Feb=160 Mar=20
</commit_message>
<xml_diff>
--- a/Reporte_Gastos_Tecnologia_Bolivar_2026.xlsx
+++ b/Reporte_Gastos_Tecnologia_Bolivar_2026.xlsx
@@ -126,7 +126,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -190,11 +190,88 @@
         <color rgb="000D7A5F"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B3F6E"/>
+      </left>
+      <right style="medium">
+        <color rgb="001B3F6E"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B3F6E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B3F6E"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -272,6 +349,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -678,6 +758,34 @@
           <t>INVERSIONES BOLÍVAR S.A. DE C.V.  ·  PRESUPUESTO ÁREA DE TECNOLOGÍA 2026</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="27" t="n"/>
+      <c r="K1" s="27" t="n"/>
+      <c r="L1" s="27" t="n"/>
+      <c r="M1" s="27" t="n"/>
+      <c r="N1" s="27" t="n"/>
+      <c r="O1" s="27" t="n"/>
+      <c r="P1" s="27" t="n"/>
+      <c r="Q1" s="27" t="n"/>
+      <c r="R1" s="27" t="n"/>
+      <c r="S1" s="27" t="n"/>
+      <c r="T1" s="27" t="n"/>
+      <c r="U1" s="27" t="n"/>
+      <c r="V1" s="27" t="n"/>
+      <c r="W1" s="27" t="n"/>
+      <c r="X1" s="27" t="n"/>
+      <c r="Y1" s="27" t="n"/>
+      <c r="Z1" s="27" t="n"/>
+      <c r="AA1" s="27" t="n"/>
+      <c r="AB1" s="27" t="n"/>
+      <c r="AC1" s="28" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -685,6 +793,34 @@
           <t>Seguimiento Presupuestal — Ppto vs Real por partida y proveedor</t>
         </is>
       </c>
+      <c r="B2" s="27" t="n"/>
+      <c r="C2" s="27" t="n"/>
+      <c r="D2" s="27" t="n"/>
+      <c r="E2" s="27" t="n"/>
+      <c r="F2" s="27" t="n"/>
+      <c r="G2" s="27" t="n"/>
+      <c r="H2" s="27" t="n"/>
+      <c r="I2" s="27" t="n"/>
+      <c r="J2" s="27" t="n"/>
+      <c r="K2" s="27" t="n"/>
+      <c r="L2" s="27" t="n"/>
+      <c r="M2" s="27" t="n"/>
+      <c r="N2" s="27" t="n"/>
+      <c r="O2" s="27" t="n"/>
+      <c r="P2" s="27" t="n"/>
+      <c r="Q2" s="27" t="n"/>
+      <c r="R2" s="27" t="n"/>
+      <c r="S2" s="27" t="n"/>
+      <c r="T2" s="27" t="n"/>
+      <c r="U2" s="27" t="n"/>
+      <c r="V2" s="27" t="n"/>
+      <c r="W2" s="27" t="n"/>
+      <c r="X2" s="27" t="n"/>
+      <c r="Y2" s="27" t="n"/>
+      <c r="Z2" s="27" t="n"/>
+      <c r="AA2" s="27" t="n"/>
+      <c r="AB2" s="27" t="n"/>
+      <c r="AC2" s="28" t="n"/>
     </row>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -692,6 +828,34 @@
           <t>Fuente: PPTO Josué &amp; Judith + Intelisis ERP (DatGastosConta)  ·  28/05/2026</t>
         </is>
       </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="27" t="n"/>
+      <c r="J3" s="27" t="n"/>
+      <c r="K3" s="27" t="n"/>
+      <c r="L3" s="27" t="n"/>
+      <c r="M3" s="27" t="n"/>
+      <c r="N3" s="27" t="n"/>
+      <c r="O3" s="27" t="n"/>
+      <c r="P3" s="27" t="n"/>
+      <c r="Q3" s="27" t="n"/>
+      <c r="R3" s="27" t="n"/>
+      <c r="S3" s="27" t="n"/>
+      <c r="T3" s="27" t="n"/>
+      <c r="U3" s="27" t="n"/>
+      <c r="V3" s="27" t="n"/>
+      <c r="W3" s="27" t="n"/>
+      <c r="X3" s="27" t="n"/>
+      <c r="Y3" s="27" t="n"/>
+      <c r="Z3" s="27" t="n"/>
+      <c r="AA3" s="27" t="n"/>
+      <c r="AB3" s="27" t="n"/>
+      <c r="AC3" s="28" t="n"/>
     </row>
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="20" customHeight="1">
@@ -710,61 +874,73 @@
           <t>Ene</t>
         </is>
       </c>
+      <c r="D5" s="28" t="n"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
+      <c r="F5" s="28" t="n"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
+      <c r="H5" s="28" t="n"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Abr</t>
         </is>
       </c>
+      <c r="J5" s="28" t="n"/>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
+      <c r="L5" s="28" t="n"/>
       <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
+      <c r="N5" s="28" t="n"/>
       <c r="O5" s="4" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
+      <c r="P5" s="28" t="n"/>
       <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>Ago</t>
         </is>
       </c>
+      <c r="R5" s="28" t="n"/>
       <c r="S5" s="4" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
+      <c r="T5" s="28" t="n"/>
       <c r="U5" s="4" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
+      <c r="V5" s="28" t="n"/>
       <c r="W5" s="4" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
+      <c r="X5" s="28" t="n"/>
       <c r="Y5" s="4" t="inlineStr">
         <is>
           <t>Dic</t>
         </is>
       </c>
+      <c r="Z5" s="28" t="n"/>
       <c r="AA5" s="4" t="inlineStr">
         <is>
           <t>Total Ppto</t>
@@ -782,6 +958,8 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="29" t="n"/>
+      <c r="B6" s="29" t="n"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Ppto</t>
@@ -902,6 +1080,9 @@
           <t>Real</t>
         </is>
       </c>
+      <c r="AA6" s="29" t="n"/>
+      <c r="AB6" s="29" t="n"/>
+      <c r="AC6" s="29" t="n"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -3645,12 +3826,12 @@
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>ADM-SUSCRIPCIONES Y PUBLICACIONES</t>
+          <t>UDESA-SUSCRIPCIONES DE SOFTWARE</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>OpenAI ChatGPT Plus — múltiples usuarios / CC</t>
+          <t>OpenAI ChatGPT Plus — mult. usuarios (CC20/40/50/410)</t>
         </is>
       </c>
       <c r="C54" s="15" t="n"/>
@@ -3659,14 +3840,14 @@
       </c>
       <c r="E54" s="15" t="n"/>
       <c r="F54" s="17" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="G54" s="15" t="n"/>
       <c r="H54" s="17" t="n">
         <v>20</v>
       </c>
       <c r="I54" s="15" t="n"/>
-      <c r="J54" s="9" t="n"/>
+      <c r="J54" s="15" t="n"/>
       <c r="K54" s="15" t="n"/>
       <c r="L54" s="9" t="n"/>
       <c r="M54" s="15" t="n"/>
@@ -3683,7 +3864,9 @@
       <c r="X54" s="9" t="n"/>
       <c r="Y54" s="15" t="n"/>
       <c r="Z54" s="9" t="n"/>
-      <c r="AA54" s="19" t="n"/>
+      <c r="AA54" s="18" t="n">
+        <v>240</v>
+      </c>
       <c r="AB54" s="18" t="n">
         <v>220</v>
       </c>
@@ -3699,6 +3882,7 @@
           <t>TOTAL GENERAL — 48 partidas</t>
         </is>
       </c>
+      <c r="B55" s="28" t="n"/>
       <c r="C55" s="21" t="n">
         <v>23377.1</v>
       </c>

</xml_diff>